<commit_message>
proceedings neu gebaut (161 S.), Slices + ZIP aktualisiert, Seitenzahlen korrigiert
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
+++ b/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X51"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
     <col width="40.83203125" customWidth="1" style="5" min="1" max="1"/>
@@ -4429,6 +4429,1189 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Web-based management and analysis of nature conservation measures in Schleswig-Holstein – current developments</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Hosenfeld, Friedrich; Krüger, Kay</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_01</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O52" t="n">
+        <v>15</v>
+      </c>
+      <c r="P52" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_01.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Common and Domain-Specific Design Patterns for Mobile AR Applications to Visualize Measures on Building Facades in an Environmental Context</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Fuchs-Kittowski, Frank; Deharde, Maximilian; Starzl, David; Poppel, Marius; Burkard, Simon</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_02</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O53" t="n">
+        <v>25</v>
+      </c>
+      <c r="P53" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_02.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sustainability Context Inheritance: From Trusted Evidence to Product Sustainability Profiles in Circular Economy Decision-Making</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Koravi, Sandhya</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_03</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>35</v>
+      </c>
+      <c r="P54" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_03.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>AI model of a photovoltaic installation</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Kobiela, Paweł; Stańczak, Jarosław; Bartoszczuk, Paweł</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_04</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O55" t="n">
+        <v>47</v>
+      </c>
+      <c r="P55" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_04.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Environmentally Informed GenAI Use in ITSM: A Problem Analysis of Organisational Use-Case Decision-Making</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Koch de Souza, Larissa; Engstler, Martin</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_05</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O56" t="n">
+        <v>57</v>
+      </c>
+      <c r="P56" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_05.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Application of Artificial Intelligence in German Municipal Wastewater Facilities</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Werner, Nicole; Thimm, Heiko; Hammann, Leonie</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_06</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O57" t="n">
+        <v>67</v>
+      </c>
+      <c r="P57" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_06.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Assessing the Maturity of Sustainability-aware Data Management Strategies that minimise Data Volumes and reduce Energy Consumption: A Study Approach</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Fellinger, Engelbert</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_07</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O58" t="n">
+        <v>79</v>
+      </c>
+      <c r="P58" t="n">
+        <v>88</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_07.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Linking Water Quality to Corrosion Behaviour at Steel Sheet Pile Walls: A Machine Learning Study in the Port of Hamburg</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Flohr, Sarah; Bruck, Paul; Kleinmann, Jan; Behrens, Grit; Kahlfeld, Andreas</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_08</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O59" t="n">
+        <v>89</v>
+      </c>
+      <c r="P59" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_08.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Air Quality Knowledge as a Driver of Computing Competences: An International Project-Based Learning Project</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Szałata, Łukasz; Behrens, Grit; Orłowski, Cezary; Grzeszczyk, Rafał</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_09</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O60" t="n">
+        <v>101</v>
+      </c>
+      <c r="P60" t="n">
+        <v>116</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Environmental Management Software</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_09.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Windows Integration into the Green Metrics Tool: Energy Measurement of Native Windows Applications via RAPL</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Jahns, Maximilian; Junger, Dennis; Wohlgemuth, Volker; Hoffmann, Geerd-Dietger</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_10</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O61" t="n">
+        <v>117</v>
+      </c>
+      <c r="P61" t="n">
+        <v>126</v>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_10.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Joint Evaluation of the Green Coding Roadmap Training</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Kriesing Garcia, Nick; Junger, Dennis; Wohlgemuth, Volker</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_11</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O62" t="n">
+        <v>127</v>
+      </c>
+      <c r="P62" t="n">
+        <v>140</v>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_11.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Toward a Framework for Performance and Carbon Footprint Assessment of Payment Channel Network Solutions</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Valko, Danila; Marx Gómez, Jorge</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_12</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O63" t="n">
+        <v>141</v>
+      </c>
+      <c r="P63" t="n">
+        <v>150</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_12.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Towards a Taxonomy of ICT and Software Sustainability Assessment Instruments</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Westing, Max; Naumann, Stefan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_13</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O64" t="n">
+        <v>151</v>
+      </c>
+      <c r="P64" t="n">
+        <v>161</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_13.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
proceedings nochmal gebaut (161 S.), Slices aktualisiert
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
+++ b/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X64"/>
+  <dimension ref="A1:X77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
     <col width="40.83203125" customWidth="1" style="5" min="1" max="1"/>
@@ -5612,6 +5612,1189 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Web-based management and analysis of nature conservation measures in Schleswig-Holstein – current developments</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Hosenfeld, Friedrich; Krüger, Kay</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_01</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O65" t="n">
+        <v>15</v>
+      </c>
+      <c r="P65" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_01.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Common and Domain-Specific Design Patterns for Mobile AR Applications to Visualize Measures on Building Facades in an Environmental Context</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Fuchs-Kittowski, Frank; Deharde, Maximilian; Starzl, David; Poppel, Marius; Burkard, Simon</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_02</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O66" t="n">
+        <v>25</v>
+      </c>
+      <c r="P66" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_02.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Sustainability Context Inheritance: From Trusted Evidence to Product Sustainability Profiles in Circular Economy Decision-Making</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Koravi, Sandhya</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_03</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O67" t="n">
+        <v>35</v>
+      </c>
+      <c r="P67" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_03.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>AI model of a photovoltaic installation</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Kobiela, Paweł; Stańczak, Jarosław; Bartoszczuk, Paweł</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_04</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>47</v>
+      </c>
+      <c r="P68" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_04.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Environmentally Informed GenAI Use in ITSM: A Problem Analysis of Organisational Use-Case Decision-Making</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Koch de Souza, Larissa; Engstler, Martin</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_05</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O69" t="n">
+        <v>57</v>
+      </c>
+      <c r="P69" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_05.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Application of Artificial Intelligence in German Municipal Wastewater Facilities</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Werner, Nicole; Thimm, Heiko; Hammann, Leonie</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_06</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O70" t="n">
+        <v>67</v>
+      </c>
+      <c r="P70" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_06.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Assessing the Maturity of Sustainability-aware Data Management Strategies that minimise Data Volumes and reduce Energy Consumption: A Study Approach</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Fellinger, Engelbert</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_07</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O71" t="n">
+        <v>79</v>
+      </c>
+      <c r="P71" t="n">
+        <v>88</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_07.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Linking Water Quality to Corrosion Behaviour at Steel Sheet Pile Walls: A Machine Learning Study in the Port of Hamburg</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Flohr, Sarah; Bruck, Paul; Kleinmann, Jan; Behrens, Grit; Kahlfeld, Andreas</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_08</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O72" t="n">
+        <v>89</v>
+      </c>
+      <c r="P72" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_08.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Air Quality Knowledge as a Driver of Computing Competences: An International Project-Based Learning Project</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Szałata, Łukasz; Behrens, Grit; Orłowski, Cezary; Grzeszczyk, Rafał</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_09</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O73" t="n">
+        <v>101</v>
+      </c>
+      <c r="P73" t="n">
+        <v>116</v>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Environmental Management Software</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_09.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Windows Integration into the Green Metrics Tool: Energy Measurement of Native Windows Applications via RAPL</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Jahns, Maximilian; Junger, Dennis; Wohlgemuth, Volker; Hoffmann, Geerd-Dietger</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_10</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O74" t="n">
+        <v>117</v>
+      </c>
+      <c r="P74" t="n">
+        <v>126</v>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_10.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Joint Evaluation of the Green Coding Roadmap Training</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Kriesing Garcia, Nick; Junger, Dennis; Wohlgemuth, Volker</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_11</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O75" t="n">
+        <v>127</v>
+      </c>
+      <c r="P75" t="n">
+        <v>140</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_11.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Toward a Framework for Performance and Carbon Footprint Assessment of Payment Channel Network Solutions</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Valko, Danila; Marx Gómez, Jorge</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_12</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O76" t="n">
+        <v>141</v>
+      </c>
+      <c r="P76" t="n">
+        <v>150</v>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_12.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Towards a Taxonomy of ICT and Software Sustainability Assessment Instruments</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Westing, Max; Naumann, Stefan</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_13</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O77" t="n">
+        <v>151</v>
+      </c>
+      <c r="P77" t="n">
+        <v>161</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_13.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
proceedings gebaut (159 S.), Slices + ZIP aktualisiert
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
+++ b/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X77"/>
+  <dimension ref="A1:X90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
     <col width="40.83203125" customWidth="1" style="5" min="1" max="1"/>
@@ -6795,6 +6795,1189 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Web-based management and analysis of nature conservation measures in Schleswig-Holstein – current developments</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Hosenfeld, Friedrich; Krüger, Kay</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_01</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O78" t="n">
+        <v>15</v>
+      </c>
+      <c r="P78" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_01.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Common and Domain-Specific Design Patterns for Mobile AR Applications to Visualize Measures on Building Facades in an Environmental Context</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Fuchs-Kittowski, Frank; Deharde, Maximilian; Starzl, David; Poppel, Marius; Burkard, Simon</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_02</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O79" t="n">
+        <v>25</v>
+      </c>
+      <c r="P79" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_02.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Sustainability Context Inheritance: From Trusted Evidence to Product Sustainability Profiles in Circular Economy Decision-Making</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Koravi, Sandhya</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_03</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O80" t="n">
+        <v>35</v>
+      </c>
+      <c r="P80" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Sustainable Development and Sustainability Concepts</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_03.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>AI model of a photovoltaic installation</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Kobiela, Paweł; Stańczak, Jarosław; Bartoszczuk, Paweł</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_04</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O81" t="n">
+        <v>47</v>
+      </c>
+      <c r="P81" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_04.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Environmentally Informed GenAI Use in ITSM: A Problem Analysis of Organisational Use-Case Decision-Making</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Koch de Souza, Larissa; Engstler, Martin</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_05</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O82" t="n">
+        <v>57</v>
+      </c>
+      <c r="P82" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_05.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Application of Artificial Intelligence in German Municipal Wastewater Facilities</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Werner, Nicole; Thimm, Heiko; Hammann, Leonie</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_06</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O83" t="n">
+        <v>67</v>
+      </c>
+      <c r="P83" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Sustainability</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_06.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Assessing the Maturity of Sustainability-aware Data Management Strategies that minimise Data Volumes and reduce Energy Consumption: A Study Approach</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Fellinger, Engelbert</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_07</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O84" t="n">
+        <v>79</v>
+      </c>
+      <c r="P84" t="n">
+        <v>88</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_07.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Linking Water Quality to Corrosion Behaviour at Steel Sheet Pile Walls: A Machine Learning Study in the Port of Hamburg</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Flohr, Sarah; Bruck, Paul; Kleinmann, Jan; Behrens, Grit; Kahlfeld, Andreas</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_08</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O85" t="n">
+        <v>89</v>
+      </c>
+      <c r="P85" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Doctoral Workshop</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_08.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Air Quality Knowledge as a Driver of Computing Competences: An International Project-Based Learning Project</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Szałata, Łukasz; Behrens, Grit; Orłowski, Cezary; Grzeszczyk, Rafał</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_09</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O86" t="n">
+        <v>101</v>
+      </c>
+      <c r="P86" t="n">
+        <v>114</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Environmental Management Software</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_09.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Windows Integration into the Green Metrics Tool: Energy Measurement of Native Windows Applications via RAPL</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Jahns, Maximilian; Junger, Dennis; Wohlgemuth, Volker; Hoffmann, Geerd-Dietger</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_10</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O87" t="n">
+        <v>115</v>
+      </c>
+      <c r="P87" t="n">
+        <v>124</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_10.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Joint Evaluation of the Green Coding Roadmap Training</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Kriesing Garcia, Nick; Junger, Dennis; Wohlgemuth, Volker</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_11</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O88" t="n">
+        <v>125</v>
+      </c>
+      <c r="P88" t="n">
+        <v>138</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_11.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Toward a Framework for Performance and Carbon Footprint Assessment of Payment Channel Network Solutions</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Valko, Danila; Marx Gómez, Jorge</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_12</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O89" t="n">
+        <v>139</v>
+      </c>
+      <c r="P89" t="n">
+        <v>148</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_12.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Towards a Taxonomy of ICT and Software Sustainability Assessment Instruments</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Westing, Max; Naumann, Stefan</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>EnviroInfo 2026</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Wohlgemuth, Volker; Wohlgemuth, Hendrik; Junger, Dennis</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Lecture Notes in Informatics (LNI) - Proceedings</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Gesellschaft für Informatik e.V.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Bonn</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>10.18420/env2026_13</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>2944-7682</t>
+        </is>
+      </c>
+      <c r="O90" t="n">
+        <v>149</v>
+      </c>
+      <c r="P90" t="n">
+        <v>159</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>09.-11. September 2026</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Bochum, Germany</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Green Coding</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Text/Conference Paper</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>10.18420-env2026_13.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>